<commit_message>
added survival to ploidy correlation
</commit_message>
<xml_diff>
--- a/data/ploidy/field/ploidy_field_performance.xlsx
+++ b/data/ploidy/field/ploidy_field_performance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ashuffmyer/MyProjects/oysters/vims-resazurin/data/ploidy/field/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A55F7187-1A3B-ED46-AE0A-6E0F5CED7E7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ABA21C6-97DD-694E-9D29-B17FD4F70E92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51480" yWindow="-1460" windowWidth="17020" windowHeight="19980" xr2:uid="{9506B5CE-A628-164C-A7D7-A7FBD8EB9181}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17760" xr2:uid="{9506B5CE-A628-164C-A7D7-A7FBD8EB9181}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1070" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="912" uniqueCount="80">
   <si>
     <t>date</t>
   </si>
@@ -254,12 +254,6 @@
     <t>found dead during tagging, but clearly dead befoe assay</t>
   </si>
   <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
     <t>tag</t>
   </si>
   <si>
@@ -390,7 +384,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -410,7 +404,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -790,50 +783,50 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
+        <v>66</v>
+      </c>
+      <c r="H1" t="s">
+        <v>71</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="M1" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="H1" t="s">
-        <v>73</v>
-      </c>
-      <c r="I1" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="J1" s="11" t="s">
+      <c r="N1" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="O1" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="P1" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="Q1" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="R1" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="S1" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="T1" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="N1" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="O1" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="P1" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q1" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="R1" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="S1" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="T1" s="9" t="s">
-        <v>72</v>
-      </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A2" s="13">
+      <c r="A2">
         <v>20250826</v>
       </c>
       <c r="B2" t="s">
@@ -854,8 +847,8 @@
       <c r="G2">
         <v>500</v>
       </c>
-      <c r="H2" t="s">
-        <v>67</v>
+      <c r="H2">
+        <v>0</v>
       </c>
       <c r="I2" s="5">
         <v>63.53</v>
@@ -892,7 +885,7 @@
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A3" s="13">
+      <c r="A3">
         <v>20250826</v>
       </c>
       <c r="B3" t="s">
@@ -913,8 +906,8 @@
       <c r="G3">
         <v>501</v>
       </c>
-      <c r="H3" t="s">
-        <v>67</v>
+      <c r="H3">
+        <v>0</v>
       </c>
       <c r="I3" s="5">
         <v>57.63</v>
@@ -951,7 +944,7 @@
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A4" s="13">
+      <c r="A4">
         <v>20250826</v>
       </c>
       <c r="B4" t="s">
@@ -972,8 +965,8 @@
       <c r="G4">
         <v>502</v>
       </c>
-      <c r="H4" t="s">
-        <v>67</v>
+      <c r="H4">
+        <v>0</v>
       </c>
       <c r="I4" s="5">
         <v>67.94</v>
@@ -1010,7 +1003,7 @@
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A5" s="13">
+      <c r="A5">
         <v>20250826</v>
       </c>
       <c r="B5" t="s">
@@ -1031,8 +1024,8 @@
       <c r="G5">
         <v>503</v>
       </c>
-      <c r="H5" t="s">
-        <v>67</v>
+      <c r="H5">
+        <v>0</v>
       </c>
       <c r="I5" s="5">
         <v>66.19</v>
@@ -1069,7 +1062,7 @@
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A6" s="13">
+      <c r="A6">
         <v>20250826</v>
       </c>
       <c r="B6" t="s">
@@ -1090,8 +1083,8 @@
       <c r="G6">
         <v>504</v>
       </c>
-      <c r="H6" t="s">
-        <v>67</v>
+      <c r="H6">
+        <v>0</v>
       </c>
       <c r="I6" s="5">
         <v>65.239999999999995</v>
@@ -1128,7 +1121,7 @@
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A7" s="13">
+      <c r="A7">
         <v>20250826</v>
       </c>
       <c r="B7" t="s">
@@ -1149,8 +1142,8 @@
       <c r="G7">
         <v>505</v>
       </c>
-      <c r="H7" t="s">
-        <v>67</v>
+      <c r="H7">
+        <v>0</v>
       </c>
       <c r="I7" s="5">
         <v>64.89</v>
@@ -1187,7 +1180,7 @@
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A8" s="13">
+      <c r="A8">
         <v>20250826</v>
       </c>
       <c r="B8" t="s">
@@ -1208,15 +1201,15 @@
       <c r="G8">
         <v>506</v>
       </c>
-      <c r="H8" t="s">
-        <v>66</v>
+      <c r="H8">
+        <v>1</v>
       </c>
       <c r="I8">
         <v>48.45</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A9" s="13">
+      <c r="A9">
         <v>20250826</v>
       </c>
       <c r="B9" t="s">
@@ -1237,8 +1230,8 @@
       <c r="G9">
         <v>507</v>
       </c>
-      <c r="H9" t="s">
-        <v>67</v>
+      <c r="H9">
+        <v>0</v>
       </c>
       <c r="I9">
         <v>75.62</v>
@@ -1279,7 +1272,7 @@
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A10" s="13">
+      <c r="A10">
         <v>20250826</v>
       </c>
       <c r="B10" t="s">
@@ -1300,8 +1293,8 @@
       <c r="G10">
         <v>508</v>
       </c>
-      <c r="H10" t="s">
-        <v>67</v>
+      <c r="H10">
+        <v>0</v>
       </c>
       <c r="I10">
         <v>65.67</v>
@@ -1342,7 +1335,7 @@
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A11" s="13">
+      <c r="A11">
         <v>20250826</v>
       </c>
       <c r="B11" t="s">
@@ -1363,8 +1356,8 @@
       <c r="G11">
         <v>509</v>
       </c>
-      <c r="H11" t="s">
-        <v>67</v>
+      <c r="H11">
+        <v>0</v>
       </c>
       <c r="I11">
         <v>61.82</v>
@@ -1405,7 +1398,7 @@
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A12" s="13">
+      <c r="A12">
         <v>20250826</v>
       </c>
       <c r="B12" t="s">
@@ -1429,7 +1422,7 @@
       <c r="H12" s="12"/>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A13" s="13">
+      <c r="A13">
         <v>20250826</v>
       </c>
       <c r="B13" t="s">
@@ -1450,8 +1443,8 @@
       <c r="G13">
         <v>511</v>
       </c>
-      <c r="H13" t="s">
-        <v>67</v>
+      <c r="H13">
+        <v>0</v>
       </c>
       <c r="I13">
         <v>71.069999999999993</v>
@@ -1492,7 +1485,7 @@
       </c>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A14" s="13">
+      <c r="A14">
         <v>20250826</v>
       </c>
       <c r="B14" t="s">
@@ -1513,8 +1506,8 @@
       <c r="G14">
         <v>512</v>
       </c>
-      <c r="H14" t="s">
-        <v>67</v>
+      <c r="H14">
+        <v>0</v>
       </c>
       <c r="I14">
         <v>57.67</v>
@@ -1555,7 +1548,7 @@
       </c>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A15" s="13">
+      <c r="A15">
         <v>20250826</v>
       </c>
       <c r="B15" t="s">
@@ -1576,8 +1569,8 @@
       <c r="G15">
         <v>513</v>
       </c>
-      <c r="H15" t="s">
-        <v>67</v>
+      <c r="H15">
+        <v>0</v>
       </c>
       <c r="I15">
         <v>54.03</v>
@@ -1618,7 +1611,7 @@
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A16" s="13">
+      <c r="A16">
         <v>20250826</v>
       </c>
       <c r="B16" t="s">
@@ -1639,12 +1632,12 @@
       <c r="G16">
         <v>514</v>
       </c>
-      <c r="H16" t="s">
-        <v>66</v>
+      <c r="H16">
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A17" s="13">
+      <c r="A17">
         <v>20250826</v>
       </c>
       <c r="B17" t="s">
@@ -1665,8 +1658,8 @@
       <c r="G17">
         <v>515</v>
       </c>
-      <c r="H17" t="s">
-        <v>67</v>
+      <c r="H17">
+        <v>0</v>
       </c>
       <c r="I17">
         <v>55.23</v>
@@ -1702,12 +1695,12 @@
         <v>1.2349999999999999</v>
       </c>
       <c r="S17" s="6">
-        <f>(R17/(N17-O17))*100</f>
+        <f t="shared" ref="S17:S23" si="3">(R17/(N17-O17))*100</f>
         <v>7.1610808303374682</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A18" s="13">
+      <c r="A18">
         <v>20250826</v>
       </c>
       <c r="B18" t="s">
@@ -1728,8 +1721,8 @@
       <c r="G18">
         <v>516</v>
       </c>
-      <c r="H18" t="s">
-        <v>67</v>
+      <c r="H18">
+        <v>0</v>
       </c>
       <c r="I18">
         <v>56.72</v>
@@ -1765,12 +1758,12 @@
         <v>0.96499999999999986</v>
       </c>
       <c r="S18" s="6">
-        <f>(R18/(N18-O18))*100</f>
+        <f t="shared" si="3"/>
         <v>7.057704965991368</v>
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A19" s="13">
+      <c r="A19">
         <v>20250826</v>
       </c>
       <c r="B19" t="s">
@@ -1791,8 +1784,8 @@
       <c r="G19">
         <v>517</v>
       </c>
-      <c r="H19" t="s">
-        <v>67</v>
+      <c r="H19">
+        <v>0</v>
       </c>
       <c r="I19">
         <v>55.2</v>
@@ -1828,12 +1821,12 @@
         <v>1.044</v>
       </c>
       <c r="S19" s="6">
-        <f>(R19/(N19-O19))*100</f>
+        <f t="shared" si="3"/>
         <v>7.7771156138259858</v>
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A20" s="13">
+      <c r="A20">
         <v>20250826</v>
       </c>
       <c r="B20" t="s">
@@ -1854,8 +1847,8 @@
       <c r="G20">
         <v>518</v>
       </c>
-      <c r="H20" t="s">
-        <v>67</v>
+      <c r="H20">
+        <v>0</v>
       </c>
       <c r="I20">
         <v>67.650000000000006</v>
@@ -1891,12 +1884,12 @@
         <v>2.7900000000000005</v>
       </c>
       <c r="S20" s="6">
-        <f>(R20/(N20-O20))*100</f>
+        <f t="shared" si="3"/>
         <v>13.209601818095734</v>
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A21" s="13">
+      <c r="A21">
         <v>20250826</v>
       </c>
       <c r="B21" t="s">
@@ -1917,8 +1910,8 @@
       <c r="G21">
         <v>519</v>
       </c>
-      <c r="H21" t="s">
-        <v>67</v>
+      <c r="H21">
+        <v>0</v>
       </c>
       <c r="I21">
         <v>68.39</v>
@@ -1954,12 +1947,12 @@
         <v>1.3460000000000001</v>
       </c>
       <c r="S21" s="6">
-        <f>(R21/(N21-O21))*100</f>
+        <f t="shared" si="3"/>
         <v>9.0713034101630949</v>
       </c>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A22" s="13">
+      <c r="A22">
         <v>20250826</v>
       </c>
       <c r="B22" t="s">
@@ -1980,8 +1973,8 @@
       <c r="G22">
         <v>520</v>
       </c>
-      <c r="H22" t="s">
-        <v>67</v>
+      <c r="H22">
+        <v>0</v>
       </c>
       <c r="I22">
         <v>71.62</v>
@@ -2017,12 +2010,12 @@
         <v>1.1280000000000001</v>
       </c>
       <c r="S22" s="6">
-        <f>(R22/(N22-O22))*100</f>
+        <f t="shared" si="3"/>
         <v>5.8640049906425471</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A23" s="13">
+      <c r="A23">
         <v>20250826</v>
       </c>
       <c r="B23" t="s">
@@ -2043,8 +2036,8 @@
       <c r="G23">
         <v>521</v>
       </c>
-      <c r="H23" t="s">
-        <v>67</v>
+      <c r="H23">
+        <v>0</v>
       </c>
       <c r="I23">
         <v>75.64</v>
@@ -2080,12 +2073,12 @@
         <v>1.157</v>
       </c>
       <c r="S23" s="6">
-        <f>(R23/(N23-O23))*100</f>
+        <f t="shared" si="3"/>
         <v>5.165870429075321</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A24" s="13">
+      <c r="A24">
         <v>20250826</v>
       </c>
       <c r="B24" t="s">
@@ -2106,15 +2099,15 @@
       <c r="G24">
         <v>522</v>
       </c>
-      <c r="H24" t="s">
-        <v>66</v>
+      <c r="H24">
+        <v>1</v>
       </c>
       <c r="I24">
         <v>47.18</v>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A25" s="13">
+      <c r="A25">
         <v>20250826</v>
       </c>
       <c r="B25" t="s">
@@ -2135,8 +2128,8 @@
       <c r="G25">
         <v>523</v>
       </c>
-      <c r="H25" t="s">
-        <v>67</v>
+      <c r="H25">
+        <v>0</v>
       </c>
       <c r="I25">
         <v>64.5</v>
@@ -2148,11 +2141,11 @@
         <v>27.63</v>
       </c>
       <c r="L25">
-        <f t="shared" ref="L25:L33" si="3">K25/I25</f>
+        <f t="shared" ref="L25:L33" si="4">K25/I25</f>
         <v>0.4283720930232558</v>
       </c>
       <c r="M25">
-        <f t="shared" ref="M25:M33" si="4">J25/I25</f>
+        <f t="shared" ref="M25:M33" si="5">J25/I25</f>
         <v>0.77519379844961245</v>
       </c>
       <c r="N25">
@@ -2168,16 +2161,16 @@
         <v>3.2170000000000001</v>
       </c>
       <c r="R25">
-        <f t="shared" ref="R25:R33" si="5">Q25-P25</f>
+        <f t="shared" ref="R25:R33" si="6">Q25-P25</f>
         <v>0.99400000000000022</v>
       </c>
       <c r="S25" s="6">
-        <f>(R25/(N25-O25))*100</f>
+        <f t="shared" ref="S25:S33" si="7">(R25/(N25-O25))*100</f>
         <v>7.2911318125137541</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A26" s="13">
+      <c r="A26">
         <v>20250826</v>
       </c>
       <c r="B26" t="s">
@@ -2198,8 +2191,8 @@
       <c r="G26">
         <v>524</v>
       </c>
-      <c r="H26" t="s">
-        <v>67</v>
+      <c r="H26">
+        <v>0</v>
       </c>
       <c r="I26">
         <v>66.650000000000006</v>
@@ -2211,11 +2204,11 @@
         <v>27.57</v>
       </c>
       <c r="L26">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.41365341335333833</v>
       </c>
       <c r="M26">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.81515378844711173</v>
       </c>
       <c r="N26">
@@ -2231,16 +2224,16 @@
         <v>4.3049999999999997</v>
       </c>
       <c r="R26">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>2.0419999999999998</v>
       </c>
       <c r="S26" s="6">
-        <f>(R26/(N26-O26))*100</f>
+        <f t="shared" si="7"/>
         <v>14.361066179056198</v>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A27" s="13">
+      <c r="A27">
         <v>20250826</v>
       </c>
       <c r="B27" t="s">
@@ -2261,8 +2254,8 @@
       <c r="G27">
         <v>525</v>
       </c>
-      <c r="H27" t="s">
-        <v>67</v>
+      <c r="H27">
+        <v>0</v>
       </c>
       <c r="I27">
         <v>67.87</v>
@@ -2274,11 +2267,11 @@
         <v>28.93</v>
       </c>
       <c r="L27">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.426256077795786</v>
       </c>
       <c r="M27">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.7901871224399587</v>
       </c>
       <c r="N27">
@@ -2294,16 +2287,16 @@
         <v>4.4020000000000001</v>
       </c>
       <c r="R27">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>2.1020000000000003</v>
       </c>
       <c r="S27" s="6">
-        <f>(R27/(N27-O27))*100</f>
+        <f t="shared" si="7"/>
         <v>9.7296796889464936</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A28" s="13">
+      <c r="A28">
         <v>20250826</v>
       </c>
       <c r="B28" t="s">
@@ -2324,8 +2317,8 @@
       <c r="G28">
         <v>526</v>
       </c>
-      <c r="H28" t="s">
-        <v>67</v>
+      <c r="H28">
+        <v>0</v>
       </c>
       <c r="I28">
         <v>63.8</v>
@@ -2337,11 +2330,11 @@
         <v>23.69</v>
       </c>
       <c r="L28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.37131661442006275</v>
       </c>
       <c r="M28">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.81771159874608157</v>
       </c>
       <c r="N28">
@@ -2357,16 +2350,16 @@
         <v>3.1669999999999998</v>
       </c>
       <c r="R28">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.94399999999999995</v>
       </c>
       <c r="S28" s="6">
-        <f>(R28/(N28-O28))*100</f>
+        <f t="shared" si="7"/>
         <v>6.9544717842935029</v>
       </c>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A29" s="13">
+      <c r="A29">
         <v>20250826</v>
       </c>
       <c r="B29" t="s">
@@ -2387,8 +2380,8 @@
       <c r="G29">
         <v>527</v>
       </c>
-      <c r="H29" t="s">
-        <v>67</v>
+      <c r="H29">
+        <v>0</v>
       </c>
       <c r="I29">
         <v>54.12</v>
@@ -2400,11 +2393,11 @@
         <v>23.8</v>
       </c>
       <c r="L29">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.4397634885439764</v>
       </c>
       <c r="M29">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.87786400591278646</v>
       </c>
       <c r="N29">
@@ -2420,16 +2413,16 @@
         <v>3.0019999999999998</v>
       </c>
       <c r="R29">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.73299999999999965</v>
       </c>
       <c r="S29" s="6">
-        <f>(R29/(N29-O29))*100</f>
+        <f t="shared" si="7"/>
         <v>6.1814808568055311</v>
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A30" s="13">
+      <c r="A30">
         <v>20250826</v>
       </c>
       <c r="B30" t="s">
@@ -2450,8 +2443,8 @@
       <c r="G30">
         <v>528</v>
       </c>
-      <c r="H30" t="s">
-        <v>67</v>
+      <c r="H30">
+        <v>0</v>
       </c>
       <c r="I30">
         <v>59.28</v>
@@ -2463,11 +2456,11 @@
         <v>29.09</v>
       </c>
       <c r="L30">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.49072199730094468</v>
       </c>
       <c r="M30">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.87246963562753033</v>
       </c>
       <c r="N30">
@@ -2483,16 +2476,16 @@
         <v>3.4409999999999998</v>
       </c>
       <c r="R30">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1.2039999999999997</v>
       </c>
       <c r="S30" s="6">
-        <f>(R30/(N30-O30))*100</f>
+        <f t="shared" si="7"/>
         <v>9.27795330199584</v>
       </c>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A31" s="13">
+      <c r="A31">
         <v>20250826</v>
       </c>
       <c r="B31" t="s">
@@ -2513,8 +2506,8 @@
       <c r="G31">
         <v>529</v>
       </c>
-      <c r="H31" t="s">
-        <v>67</v>
+      <c r="H31">
+        <v>0</v>
       </c>
       <c r="I31">
         <v>64.66</v>
@@ -2526,11 +2519,11 @@
         <v>25.22</v>
       </c>
       <c r="L31">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.39004021033096198</v>
       </c>
       <c r="M31">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.76987318280235084</v>
       </c>
       <c r="N31">
@@ -2546,16 +2539,16 @@
         <v>3.4460000000000002</v>
       </c>
       <c r="R31">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1.2110000000000003</v>
       </c>
       <c r="S31" s="6">
-        <f>(R31/(N31-O31))*100</f>
+        <f t="shared" si="7"/>
         <v>7.6480990274093736</v>
       </c>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A32" s="13">
+      <c r="A32">
         <v>20250826</v>
       </c>
       <c r="B32" t="s">
@@ -2576,8 +2569,8 @@
       <c r="G32">
         <v>530</v>
       </c>
-      <c r="H32" t="s">
-        <v>67</v>
+      <c r="H32">
+        <v>0</v>
       </c>
       <c r="I32">
         <v>79.739999999999995</v>
@@ -2589,11 +2582,11 @@
         <v>29.55</v>
       </c>
       <c r="L32">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.37057938299473292</v>
       </c>
       <c r="M32">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.76812139453222983</v>
       </c>
       <c r="N32">
@@ -2609,16 +2602,16 @@
         <v>4.7839999999999998</v>
       </c>
       <c r="R32">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>2.5469999999999997</v>
       </c>
       <c r="S32" s="6">
-        <f>(R32/(N32-O32))*100</f>
+        <f t="shared" si="7"/>
         <v>9.5683534317592684</v>
       </c>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A33" s="13">
+      <c r="A33">
         <v>20250826</v>
       </c>
       <c r="B33" t="s">
@@ -2639,8 +2632,8 @@
       <c r="G33">
         <v>531</v>
       </c>
-      <c r="H33" t="s">
-        <v>67</v>
+      <c r="H33">
+        <v>0</v>
       </c>
       <c r="I33">
         <v>70.88</v>
@@ -2652,11 +2645,11 @@
         <v>25.33</v>
       </c>
       <c r="L33">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.35736455981941312</v>
       </c>
       <c r="M33">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.76312076749435676</v>
       </c>
       <c r="N33">
@@ -2672,16 +2665,16 @@
         <v>4.17</v>
       </c>
       <c r="R33">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1.9289999999999998</v>
       </c>
       <c r="S33" s="6">
-        <f>(R33/(N33-O33))*100</f>
+        <f t="shared" si="7"/>
         <v>9.3786464410735082</v>
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A34" s="13">
+      <c r="A34">
         <v>20250826</v>
       </c>
       <c r="B34" t="s">
@@ -2705,7 +2698,7 @@
       <c r="H34" s="12"/>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A35" s="13">
+      <c r="A35">
         <v>20250826</v>
       </c>
       <c r="B35" t="s">
@@ -2726,8 +2719,8 @@
       <c r="G35">
         <v>533</v>
       </c>
-      <c r="H35" t="s">
-        <v>67</v>
+      <c r="H35">
+        <v>0</v>
       </c>
       <c r="I35">
         <v>79.25</v>
@@ -2768,7 +2761,7 @@
       </c>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A36" s="13">
+      <c r="A36">
         <v>20250826</v>
       </c>
       <c r="B36" t="s">
@@ -2789,15 +2782,15 @@
       <c r="G36">
         <v>534</v>
       </c>
-      <c r="H36" t="s">
-        <v>66</v>
+      <c r="H36">
+        <v>1</v>
       </c>
       <c r="I36">
         <v>88.66</v>
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A37" s="13">
+      <c r="A37">
         <v>20250826</v>
       </c>
       <c r="B37" t="s">
@@ -2818,8 +2811,8 @@
       <c r="G37">
         <v>535</v>
       </c>
-      <c r="H37" t="s">
-        <v>67</v>
+      <c r="H37">
+        <v>0</v>
       </c>
       <c r="I37">
         <v>56.07</v>
@@ -2860,7 +2853,7 @@
       </c>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A38" s="13">
+      <c r="A38">
         <v>20250826</v>
       </c>
       <c r="B38" t="s">
@@ -2881,12 +2874,12 @@
       <c r="G38">
         <v>536</v>
       </c>
-      <c r="H38" t="s">
-        <v>66</v>
+      <c r="H38">
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A39" s="13">
+      <c r="A39">
         <v>20250826</v>
       </c>
       <c r="B39" t="s">
@@ -2907,8 +2900,8 @@
       <c r="G39">
         <v>537</v>
       </c>
-      <c r="H39" t="s">
-        <v>67</v>
+      <c r="H39">
+        <v>0</v>
       </c>
       <c r="I39">
         <v>47.31</v>
@@ -2949,7 +2942,7 @@
       </c>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A40" s="13">
+      <c r="A40">
         <v>20250826</v>
       </c>
       <c r="B40" t="s">
@@ -2970,8 +2963,8 @@
       <c r="G40">
         <v>538</v>
       </c>
-      <c r="H40" t="s">
-        <v>67</v>
+      <c r="H40">
+        <v>0</v>
       </c>
       <c r="I40">
         <v>69.180000000000007</v>
@@ -3012,7 +3005,7 @@
       </c>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A41" s="13">
+      <c r="A41">
         <v>20250826</v>
       </c>
       <c r="B41" t="s">
@@ -3033,8 +3026,8 @@
       <c r="G41">
         <v>539</v>
       </c>
-      <c r="H41" t="s">
-        <v>67</v>
+      <c r="H41">
+        <v>0</v>
       </c>
       <c r="I41">
         <v>62.48</v>
@@ -3075,7 +3068,7 @@
       </c>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A42" s="13">
+      <c r="A42">
         <v>20250826</v>
       </c>
       <c r="B42" t="s">
@@ -3096,8 +3089,8 @@
       <c r="G42">
         <v>540</v>
       </c>
-      <c r="H42" t="s">
-        <v>66</v>
+      <c r="H42">
+        <v>1</v>
       </c>
       <c r="I42">
         <v>49.49</v>
@@ -3105,7 +3098,7 @@
       <c r="S42" s="6"/>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A43" s="13">
+      <c r="A43">
         <v>20250826</v>
       </c>
       <c r="B43" t="s">
@@ -3126,8 +3119,8 @@
       <c r="G43">
         <v>541</v>
       </c>
-      <c r="H43" t="s">
-        <v>67</v>
+      <c r="H43">
+        <v>0</v>
       </c>
       <c r="I43">
         <v>62.95</v>
@@ -3168,7 +3161,7 @@
       </c>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A44" s="13">
+      <c r="A44">
         <v>20250826</v>
       </c>
       <c r="B44" t="s">
@@ -3189,8 +3182,8 @@
       <c r="G44">
         <v>542</v>
       </c>
-      <c r="H44" t="s">
-        <v>67</v>
+      <c r="H44">
+        <v>0</v>
       </c>
       <c r="I44">
         <v>80.930000000000007</v>
@@ -3231,7 +3224,7 @@
       </c>
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A45" s="13">
+      <c r="A45">
         <v>20250826</v>
       </c>
       <c r="B45" t="s">
@@ -3252,8 +3245,8 @@
       <c r="G45">
         <v>543</v>
       </c>
-      <c r="H45" t="s">
-        <v>67</v>
+      <c r="H45">
+        <v>0</v>
       </c>
       <c r="I45">
         <v>69.819999999999993</v>
@@ -3294,7 +3287,7 @@
       </c>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A46" s="13">
+      <c r="A46">
         <v>20250826</v>
       </c>
       <c r="B46" t="s">
@@ -3315,15 +3308,15 @@
       <c r="G46">
         <v>544</v>
       </c>
-      <c r="H46" t="s">
-        <v>66</v>
+      <c r="H46">
+        <v>1</v>
       </c>
       <c r="I46">
         <v>63.13</v>
       </c>
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A47" s="13">
+      <c r="A47">
         <v>20250826</v>
       </c>
       <c r="B47" t="s">
@@ -3344,8 +3337,8 @@
       <c r="G47">
         <v>545</v>
       </c>
-      <c r="H47" t="s">
-        <v>67</v>
+      <c r="H47">
+        <v>0</v>
       </c>
       <c r="I47">
         <v>73.64</v>
@@ -3386,7 +3379,7 @@
       </c>
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A48" s="13">
+      <c r="A48">
         <v>20250826</v>
       </c>
       <c r="B48" t="s">
@@ -3407,15 +3400,15 @@
       <c r="G48">
         <v>546</v>
       </c>
-      <c r="H48" t="s">
-        <v>66</v>
+      <c r="H48">
+        <v>1</v>
       </c>
       <c r="I48">
         <v>68.540000000000006</v>
       </c>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A49" s="13">
+      <c r="A49">
         <v>20250826</v>
       </c>
       <c r="B49" t="s">
@@ -3436,8 +3429,8 @@
       <c r="G49">
         <v>547</v>
       </c>
-      <c r="H49" t="s">
-        <v>67</v>
+      <c r="H49">
+        <v>0</v>
       </c>
       <c r="I49">
         <v>71.66</v>
@@ -3478,7 +3471,7 @@
       </c>
     </row>
     <row r="50" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A50" s="13">
+      <c r="A50">
         <v>20250826</v>
       </c>
       <c r="B50" t="s">
@@ -3499,8 +3492,8 @@
       <c r="G50">
         <v>548</v>
       </c>
-      <c r="H50" t="s">
-        <v>67</v>
+      <c r="H50">
+        <v>0</v>
       </c>
       <c r="I50">
         <v>54.83</v>
@@ -3541,7 +3534,7 @@
       </c>
     </row>
     <row r="51" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A51" s="13">
+      <c r="A51">
         <v>20250826</v>
       </c>
       <c r="B51" t="s">
@@ -3562,8 +3555,8 @@
       <c r="G51">
         <v>549</v>
       </c>
-      <c r="H51" t="s">
-        <v>67</v>
+      <c r="H51">
+        <v>0</v>
       </c>
       <c r="I51">
         <v>57.19</v>
@@ -3604,7 +3597,7 @@
       </c>
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A52" s="13">
+      <c r="A52">
         <v>20250826</v>
       </c>
       <c r="B52" t="s">
@@ -3628,7 +3621,7 @@
       <c r="H52" s="12"/>
     </row>
     <row r="53" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A53" s="13">
+      <c r="A53">
         <v>20250826</v>
       </c>
       <c r="B53" t="s">
@@ -3649,8 +3642,8 @@
       <c r="G53">
         <v>551</v>
       </c>
-      <c r="H53" t="s">
-        <v>67</v>
+      <c r="H53">
+        <v>0</v>
       </c>
       <c r="I53">
         <v>58.55</v>
@@ -3691,7 +3684,7 @@
       </c>
     </row>
     <row r="54" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A54" s="13">
+      <c r="A54">
         <v>20250826</v>
       </c>
       <c r="B54" t="s">
@@ -3712,8 +3705,8 @@
       <c r="G54">
         <v>552</v>
       </c>
-      <c r="H54" t="s">
-        <v>67</v>
+      <c r="H54">
+        <v>0</v>
       </c>
       <c r="I54">
         <v>66.84</v>
@@ -3754,7 +3747,7 @@
       </c>
     </row>
     <row r="55" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A55" s="13">
+      <c r="A55">
         <v>20250826</v>
       </c>
       <c r="B55" t="s">
@@ -3775,8 +3768,8 @@
       <c r="G55">
         <v>553</v>
       </c>
-      <c r="H55" t="s">
-        <v>67</v>
+      <c r="H55">
+        <v>0</v>
       </c>
       <c r="I55">
         <v>54.66</v>
@@ -3817,7 +3810,7 @@
       </c>
     </row>
     <row r="56" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A56" s="13">
+      <c r="A56">
         <v>20250826</v>
       </c>
       <c r="B56" t="s">
@@ -3838,15 +3831,15 @@
       <c r="G56">
         <v>554</v>
       </c>
-      <c r="H56" t="s">
-        <v>66</v>
+      <c r="H56">
+        <v>1</v>
       </c>
       <c r="I56">
         <v>47.42</v>
       </c>
     </row>
     <row r="57" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A57" s="13">
+      <c r="A57">
         <v>20250826</v>
       </c>
       <c r="B57" t="s">
@@ -3867,8 +3860,8 @@
       <c r="G57">
         <v>555</v>
       </c>
-      <c r="H57" t="s">
-        <v>67</v>
+      <c r="H57">
+        <v>0</v>
       </c>
       <c r="I57" s="5">
         <v>79.680000000000007</v>
@@ -3905,7 +3898,7 @@
       </c>
     </row>
     <row r="58" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A58" s="13">
+      <c r="A58">
         <v>20250826</v>
       </c>
       <c r="B58" t="s">
@@ -3926,8 +3919,8 @@
       <c r="G58">
         <v>556</v>
       </c>
-      <c r="H58" t="s">
-        <v>67</v>
+      <c r="H58">
+        <v>0</v>
       </c>
       <c r="I58" s="5">
         <v>72.14</v>
@@ -3964,7 +3957,7 @@
       </c>
     </row>
     <row r="59" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A59" s="13">
+      <c r="A59">
         <v>20250826</v>
       </c>
       <c r="B59" t="s">
@@ -3985,8 +3978,8 @@
       <c r="G59">
         <v>557</v>
       </c>
-      <c r="H59" t="s">
-        <v>67</v>
+      <c r="H59">
+        <v>0</v>
       </c>
       <c r="I59" s="5">
         <v>64.39</v>
@@ -4023,7 +4016,7 @@
       </c>
     </row>
     <row r="60" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A60" s="13">
+      <c r="A60">
         <v>20250826</v>
       </c>
       <c r="B60" t="s">
@@ -4044,8 +4037,8 @@
       <c r="G60">
         <v>558</v>
       </c>
-      <c r="H60" t="s">
-        <v>67</v>
+      <c r="H60">
+        <v>0</v>
       </c>
       <c r="I60" s="5">
         <v>69.86</v>
@@ -4082,7 +4075,7 @@
       </c>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A61" s="13">
+      <c r="A61">
         <v>20250826</v>
       </c>
       <c r="B61" t="s">
@@ -4103,8 +4096,8 @@
       <c r="G61">
         <v>559</v>
       </c>
-      <c r="H61" t="s">
-        <v>67</v>
+      <c r="H61">
+        <v>0</v>
       </c>
       <c r="I61" s="5">
         <v>89.66</v>
@@ -4141,7 +4134,7 @@
       </c>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A62" s="13">
+      <c r="A62">
         <v>20250826</v>
       </c>
       <c r="B62" t="s">
@@ -4162,8 +4155,8 @@
       <c r="G62">
         <v>560</v>
       </c>
-      <c r="H62" t="s">
-        <v>67</v>
+      <c r="H62">
+        <v>0</v>
       </c>
       <c r="I62" s="5">
         <v>59.85</v>
@@ -4200,7 +4193,7 @@
       </c>
     </row>
     <row r="63" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A63" s="13">
+      <c r="A63">
         <v>20250826</v>
       </c>
       <c r="B63" t="s">
@@ -4221,8 +4214,8 @@
       <c r="G63">
         <v>561</v>
       </c>
-      <c r="H63" t="s">
-        <v>67</v>
+      <c r="H63">
+        <v>0</v>
       </c>
       <c r="I63" s="5">
         <v>69.17</v>
@@ -4259,7 +4252,7 @@
       </c>
     </row>
     <row r="64" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A64" s="13">
+      <c r="A64">
         <v>20250826</v>
       </c>
       <c r="B64" t="s">
@@ -4283,7 +4276,7 @@
       <c r="H64" s="12"/>
     </row>
     <row r="65" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A65" s="13">
+      <c r="A65">
         <v>20250826</v>
       </c>
       <c r="B65" t="s">
@@ -4304,8 +4297,8 @@
       <c r="G65">
         <v>563</v>
       </c>
-      <c r="H65" t="s">
-        <v>67</v>
+      <c r="H65">
+        <v>0</v>
       </c>
       <c r="I65">
         <v>57.53</v>
@@ -4346,7 +4339,7 @@
       </c>
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A66" s="13">
+      <c r="A66">
         <v>20250826</v>
       </c>
       <c r="B66" t="s">
@@ -4367,8 +4360,8 @@
       <c r="G66">
         <v>564</v>
       </c>
-      <c r="H66" t="s">
-        <v>67</v>
+      <c r="H66">
+        <v>0</v>
       </c>
       <c r="I66">
         <v>70.400000000000006</v>
@@ -4409,7 +4402,7 @@
       </c>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A67" s="13">
+      <c r="A67">
         <v>20250826</v>
       </c>
       <c r="B67" t="s">
@@ -4430,8 +4423,8 @@
       <c r="G67">
         <v>565</v>
       </c>
-      <c r="H67" t="s">
-        <v>67</v>
+      <c r="H67">
+        <v>0</v>
       </c>
       <c r="I67">
         <v>62.23</v>
@@ -4472,7 +4465,7 @@
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A68" s="13">
+      <c r="A68">
         <v>20250826</v>
       </c>
       <c r="B68" t="s">
@@ -4493,8 +4486,8 @@
       <c r="G68">
         <v>566</v>
       </c>
-      <c r="H68" t="s">
-        <v>67</v>
+      <c r="H68">
+        <v>0</v>
       </c>
       <c r="I68">
         <v>60.6</v>
@@ -4535,7 +4528,7 @@
       </c>
     </row>
     <row r="69" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A69" s="13">
+      <c r="A69">
         <v>20250826</v>
       </c>
       <c r="B69" t="s">
@@ -4556,8 +4549,8 @@
       <c r="G69">
         <v>567</v>
       </c>
-      <c r="H69" t="s">
-        <v>67</v>
+      <c r="H69">
+        <v>0</v>
       </c>
       <c r="I69">
         <v>64.09</v>
@@ -4598,7 +4591,7 @@
       </c>
     </row>
     <row r="70" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A70" s="13">
+      <c r="A70">
         <v>20250826</v>
       </c>
       <c r="B70" t="s">
@@ -4619,15 +4612,15 @@
       <c r="G70">
         <v>568</v>
       </c>
-      <c r="H70" t="s">
-        <v>66</v>
+      <c r="H70">
+        <v>1</v>
       </c>
       <c r="I70">
         <v>67.59</v>
       </c>
     </row>
     <row r="71" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A71" s="13">
+      <c r="A71">
         <v>20250826</v>
       </c>
       <c r="B71" t="s">
@@ -4648,8 +4641,8 @@
       <c r="G71">
         <v>569</v>
       </c>
-      <c r="H71" t="s">
-        <v>67</v>
+      <c r="H71">
+        <v>0</v>
       </c>
       <c r="I71">
         <v>77.040000000000006</v>
@@ -4690,7 +4683,7 @@
       </c>
     </row>
     <row r="72" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A72" s="13">
+      <c r="A72">
         <v>20250826</v>
       </c>
       <c r="B72" t="s">
@@ -4711,15 +4704,15 @@
       <c r="G72">
         <v>570</v>
       </c>
-      <c r="H72" t="s">
-        <v>66</v>
+      <c r="H72">
+        <v>1</v>
       </c>
       <c r="I72">
         <v>63.44</v>
       </c>
     </row>
     <row r="73" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A73" s="13">
+      <c r="A73">
         <v>20250826</v>
       </c>
       <c r="B73" t="s">
@@ -4740,8 +4733,8 @@
       <c r="G73">
         <v>571</v>
       </c>
-      <c r="H73" t="s">
-        <v>67</v>
+      <c r="H73">
+        <v>0</v>
       </c>
       <c r="I73">
         <v>60.23</v>
@@ -4782,7 +4775,7 @@
       </c>
     </row>
     <row r="74" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A74" s="13">
+      <c r="A74">
         <v>20250826</v>
       </c>
       <c r="B74" t="s">
@@ -4803,8 +4796,8 @@
       <c r="G74">
         <v>572</v>
       </c>
-      <c r="H74" t="s">
-        <v>67</v>
+      <c r="H74">
+        <v>0</v>
       </c>
       <c r="I74">
         <v>64.19</v>
@@ -4845,7 +4838,7 @@
       </c>
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A75" s="13">
+      <c r="A75">
         <v>20250826</v>
       </c>
       <c r="B75" t="s">
@@ -4866,12 +4859,12 @@
       <c r="G75">
         <v>573</v>
       </c>
-      <c r="H75" t="s">
-        <v>66</v>
+      <c r="H75">
+        <v>1</v>
       </c>
     </row>
     <row r="76" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A76" s="13">
+      <c r="A76">
         <v>20250826</v>
       </c>
       <c r="B76" t="s">
@@ -4892,8 +4885,8 @@
       <c r="G76">
         <v>574</v>
       </c>
-      <c r="H76" t="s">
-        <v>67</v>
+      <c r="H76">
+        <v>0</v>
       </c>
       <c r="I76">
         <v>69.08</v>
@@ -4934,7 +4927,7 @@
       </c>
     </row>
     <row r="77" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A77" s="13">
+      <c r="A77">
         <v>20250826</v>
       </c>
       <c r="B77" t="s">
@@ -4955,8 +4948,8 @@
       <c r="G77">
         <v>575</v>
       </c>
-      <c r="H77" t="s">
-        <v>67</v>
+      <c r="H77">
+        <v>0</v>
       </c>
       <c r="I77">
         <v>57.77</v>
@@ -4997,7 +4990,7 @@
       </c>
     </row>
     <row r="78" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A78" s="13">
+      <c r="A78">
         <v>20250826</v>
       </c>
       <c r="B78" t="s">
@@ -5018,8 +5011,8 @@
       <c r="G78">
         <v>576</v>
       </c>
-      <c r="H78" t="s">
-        <v>67</v>
+      <c r="H78">
+        <v>0</v>
       </c>
       <c r="I78">
         <v>69.53</v>
@@ -5060,7 +5053,7 @@
       </c>
     </row>
     <row r="79" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A79" s="13">
+      <c r="A79">
         <v>20250826</v>
       </c>
       <c r="B79" t="s">
@@ -5081,8 +5074,8 @@
       <c r="G79">
         <v>577</v>
       </c>
-      <c r="H79" t="s">
-        <v>67</v>
+      <c r="H79">
+        <v>0</v>
       </c>
       <c r="I79">
         <v>73.680000000000007</v>
@@ -5123,7 +5116,7 @@
       </c>
     </row>
     <row r="80" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A80" s="13">
+      <c r="A80">
         <v>20250826</v>
       </c>
       <c r="B80" t="s">
@@ -5144,8 +5137,8 @@
       <c r="G80">
         <v>578</v>
       </c>
-      <c r="H80" t="s">
-        <v>67</v>
+      <c r="H80">
+        <v>0</v>
       </c>
       <c r="I80">
         <v>69.37</v>
@@ -5186,7 +5179,7 @@
       </c>
     </row>
     <row r="81" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A81" s="13">
+      <c r="A81">
         <v>20250826</v>
       </c>
       <c r="B81" t="s">
@@ -5207,15 +5200,15 @@
       <c r="G81">
         <v>579</v>
       </c>
-      <c r="H81" t="s">
-        <v>66</v>
+      <c r="H81">
+        <v>1</v>
       </c>
       <c r="I81">
         <v>50.9</v>
       </c>
     </row>
     <row r="82" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A82" s="13">
+      <c r="A82">
         <v>20250826</v>
       </c>
       <c r="B82" t="s">
@@ -5236,12 +5229,12 @@
       <c r="G82">
         <v>580</v>
       </c>
-      <c r="H82" t="s">
-        <v>66</v>
+      <c r="H82">
+        <v>1</v>
       </c>
     </row>
     <row r="83" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A83" s="13">
+      <c r="A83">
         <v>20250826</v>
       </c>
       <c r="B83" t="s">
@@ -5262,15 +5255,15 @@
       <c r="G83">
         <v>581</v>
       </c>
-      <c r="H83" t="s">
-        <v>66</v>
+      <c r="H83">
+        <v>1</v>
       </c>
       <c r="I83">
         <v>60.98</v>
       </c>
     </row>
     <row r="84" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A84" s="13">
+      <c r="A84">
         <v>20250826</v>
       </c>
       <c r="B84" t="s">
@@ -5291,8 +5284,8 @@
       <c r="G84">
         <v>582</v>
       </c>
-      <c r="H84" t="s">
-        <v>67</v>
+      <c r="H84">
+        <v>0</v>
       </c>
       <c r="I84">
         <v>75.13</v>
@@ -5333,7 +5326,7 @@
       </c>
     </row>
     <row r="85" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A85" s="13">
+      <c r="A85">
         <v>20250826</v>
       </c>
       <c r="B85" t="s">
@@ -5354,15 +5347,15 @@
       <c r="G85">
         <v>583</v>
       </c>
-      <c r="H85" t="s">
-        <v>66</v>
+      <c r="H85">
+        <v>1</v>
       </c>
       <c r="I85">
         <v>71.62</v>
       </c>
     </row>
     <row r="86" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A86" s="13">
+      <c r="A86">
         <v>20250826</v>
       </c>
       <c r="B86" t="s">
@@ -5383,8 +5376,8 @@
       <c r="G86">
         <v>584</v>
       </c>
-      <c r="H86" t="s">
-        <v>67</v>
+      <c r="H86">
+        <v>0</v>
       </c>
       <c r="I86">
         <v>64.959999999999994</v>
@@ -5425,7 +5418,7 @@
       </c>
     </row>
     <row r="87" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A87" s="13">
+      <c r="A87">
         <v>20250826</v>
       </c>
       <c r="B87" t="s">
@@ -5446,8 +5439,8 @@
       <c r="G87">
         <v>585</v>
       </c>
-      <c r="H87" t="s">
-        <v>67</v>
+      <c r="H87">
+        <v>0</v>
       </c>
       <c r="I87">
         <v>71.25</v>
@@ -5488,7 +5481,7 @@
       </c>
     </row>
     <row r="88" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A88" s="13">
+      <c r="A88">
         <v>20250826</v>
       </c>
       <c r="B88" t="s">
@@ -5512,7 +5505,7 @@
       <c r="H88" s="12"/>
     </row>
     <row r="89" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A89" s="13">
+      <c r="A89">
         <v>20250826</v>
       </c>
       <c r="B89" t="s">
@@ -5533,15 +5526,15 @@
       <c r="G89">
         <v>587</v>
       </c>
-      <c r="H89" t="s">
-        <v>66</v>
+      <c r="H89">
+        <v>1</v>
       </c>
       <c r="I89">
         <v>51.56</v>
       </c>
     </row>
     <row r="90" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A90" s="13">
+      <c r="A90">
         <v>20250826</v>
       </c>
       <c r="B90" t="s">
@@ -5562,15 +5555,15 @@
       <c r="G90">
         <v>588</v>
       </c>
-      <c r="H90" t="s">
-        <v>66</v>
+      <c r="H90">
+        <v>1</v>
       </c>
       <c r="I90">
         <v>68.48</v>
       </c>
     </row>
     <row r="91" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A91" s="13">
+      <c r="A91">
         <v>20250826</v>
       </c>
       <c r="B91" t="s">
@@ -5591,8 +5584,8 @@
       <c r="G91">
         <v>589</v>
       </c>
-      <c r="H91" t="s">
-        <v>67</v>
+      <c r="H91">
+        <v>0</v>
       </c>
       <c r="I91">
         <v>59.99</v>
@@ -5633,7 +5626,7 @@
       </c>
     </row>
     <row r="92" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A92" s="13">
+      <c r="A92">
         <v>20250826</v>
       </c>
       <c r="B92" t="s">
@@ -5654,8 +5647,8 @@
       <c r="G92">
         <v>590</v>
       </c>
-      <c r="H92" t="s">
-        <v>67</v>
+      <c r="H92">
+        <v>0</v>
       </c>
       <c r="I92">
         <v>57.41</v>
@@ -5696,7 +5689,7 @@
       </c>
     </row>
     <row r="93" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A93" s="13">
+      <c r="A93">
         <v>20250826</v>
       </c>
       <c r="B93" t="s">
@@ -5717,15 +5710,15 @@
       <c r="G93">
         <v>591</v>
       </c>
-      <c r="H93" t="s">
-        <v>66</v>
+      <c r="H93">
+        <v>1</v>
       </c>
       <c r="I93">
         <v>39.85</v>
       </c>
     </row>
     <row r="94" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A94" s="13">
+      <c r="A94">
         <v>20250826</v>
       </c>
       <c r="B94" t="s">
@@ -5746,8 +5739,8 @@
       <c r="G94">
         <v>592</v>
       </c>
-      <c r="H94" t="s">
-        <v>67</v>
+      <c r="H94">
+        <v>0</v>
       </c>
       <c r="I94">
         <v>56.27</v>
@@ -5788,7 +5781,7 @@
       </c>
     </row>
     <row r="95" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A95" s="13">
+      <c r="A95">
         <v>20250826</v>
       </c>
       <c r="B95" t="s">
@@ -5809,8 +5802,8 @@
       <c r="G95">
         <v>593</v>
       </c>
-      <c r="H95" t="s">
-        <v>67</v>
+      <c r="H95">
+        <v>0</v>
       </c>
       <c r="I95">
         <v>70.19</v>
@@ -5851,7 +5844,7 @@
       </c>
     </row>
     <row r="96" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A96" s="13">
+      <c r="A96">
         <v>20250826</v>
       </c>
       <c r="B96" t="s">
@@ -5872,8 +5865,8 @@
       <c r="G96">
         <v>594</v>
       </c>
-      <c r="H96" t="s">
-        <v>67</v>
+      <c r="H96">
+        <v>0</v>
       </c>
       <c r="I96">
         <v>63.99</v>
@@ -5914,7 +5907,7 @@
       </c>
     </row>
     <row r="97" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A97" s="13">
+      <c r="A97">
         <v>20250826</v>
       </c>
       <c r="B97" t="s">
@@ -5935,8 +5928,8 @@
       <c r="G97">
         <v>595</v>
       </c>
-      <c r="H97" t="s">
-        <v>67</v>
+      <c r="H97">
+        <v>0</v>
       </c>
       <c r="I97">
         <v>61.24</v>
@@ -5977,7 +5970,7 @@
       </c>
     </row>
     <row r="98" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A98" s="13">
+      <c r="A98">
         <v>20250826</v>
       </c>
       <c r="B98" t="s">
@@ -5998,15 +5991,15 @@
       <c r="G98">
         <v>596</v>
       </c>
-      <c r="H98" t="s">
-        <v>66</v>
+      <c r="H98">
+        <v>1</v>
       </c>
       <c r="I98">
         <v>71.62</v>
       </c>
     </row>
     <row r="99" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A99" s="13">
+      <c r="A99">
         <v>20250826</v>
       </c>
       <c r="B99" t="s">
@@ -6027,8 +6020,8 @@
       <c r="G99">
         <v>597</v>
       </c>
-      <c r="H99" t="s">
-        <v>67</v>
+      <c r="H99">
+        <v>0</v>
       </c>
       <c r="I99">
         <v>64.97</v>
@@ -6069,7 +6062,7 @@
       </c>
     </row>
     <row r="100" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A100" s="13">
+      <c r="A100">
         <v>20250826</v>
       </c>
       <c r="B100" t="s">
@@ -6090,8 +6083,8 @@
       <c r="G100">
         <v>598</v>
       </c>
-      <c r="H100" t="s">
-        <v>67</v>
+      <c r="H100">
+        <v>0</v>
       </c>
       <c r="I100">
         <v>80.95</v>
@@ -6132,7 +6125,7 @@
       </c>
     </row>
     <row r="101" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A101" s="13">
+      <c r="A101">
         <v>20250826</v>
       </c>
       <c r="B101" t="s">
@@ -6153,8 +6146,8 @@
       <c r="G101">
         <v>599</v>
       </c>
-      <c r="H101" t="s">
-        <v>67</v>
+      <c r="H101">
+        <v>0</v>
       </c>
       <c r="I101">
         <v>56.35</v>
@@ -6195,7 +6188,7 @@
       </c>
     </row>
     <row r="102" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A102" s="13">
+      <c r="A102">
         <v>20250826</v>
       </c>
       <c r="B102" t="s">
@@ -6216,8 +6209,8 @@
       <c r="G102">
         <v>600</v>
       </c>
-      <c r="H102" t="s">
-        <v>67</v>
+      <c r="H102">
+        <v>0</v>
       </c>
       <c r="I102">
         <v>71.41</v>
@@ -6258,7 +6251,7 @@
       </c>
     </row>
     <row r="103" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A103" s="13">
+      <c r="A103">
         <v>20250826</v>
       </c>
       <c r="B103" t="s">
@@ -6279,15 +6272,15 @@
       <c r="G103">
         <v>601</v>
       </c>
-      <c r="H103" t="s">
-        <v>66</v>
+      <c r="H103">
+        <v>1</v>
       </c>
       <c r="I103">
         <v>68.790000000000006</v>
       </c>
     </row>
     <row r="104" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A104" s="13">
+      <c r="A104">
         <v>20250826</v>
       </c>
       <c r="B104" t="s">
@@ -6308,15 +6301,15 @@
       <c r="G104">
         <v>602</v>
       </c>
-      <c r="H104" t="s">
-        <v>66</v>
+      <c r="H104">
+        <v>1</v>
       </c>
       <c r="I104">
         <v>60.31</v>
       </c>
     </row>
     <row r="105" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A105" s="13">
+      <c r="A105">
         <v>20250826</v>
       </c>
       <c r="B105" t="s">
@@ -6337,8 +6330,8 @@
       <c r="G105">
         <v>603</v>
       </c>
-      <c r="H105" t="s">
-        <v>67</v>
+      <c r="H105">
+        <v>0</v>
       </c>
       <c r="I105">
         <v>56.77</v>
@@ -6374,12 +6367,12 @@
         <v>1.0840000000000001</v>
       </c>
       <c r="S105" s="6">
-        <f>(R105/(N105-O105))*100</f>
+        <f t="shared" ref="S105:S120" si="8">(R105/(N105-O105))*100</f>
         <v>9.1569521878695728</v>
       </c>
     </row>
     <row r="106" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A106" s="13">
+      <c r="A106">
         <v>20250826</v>
       </c>
       <c r="B106" t="s">
@@ -6400,8 +6393,8 @@
       <c r="G106">
         <v>604</v>
       </c>
-      <c r="H106" t="s">
-        <v>67</v>
+      <c r="H106">
+        <v>0</v>
       </c>
       <c r="I106">
         <v>64.86</v>
@@ -6437,12 +6430,12 @@
         <v>1.2000000000000002</v>
       </c>
       <c r="S106" s="6">
-        <f>(R106/(N106-O106))*100</f>
+        <f t="shared" si="8"/>
         <v>5.608000747733433</v>
       </c>
     </row>
     <row r="107" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A107" s="13">
+      <c r="A107">
         <v>20250826</v>
       </c>
       <c r="B107" t="s">
@@ -6463,8 +6456,8 @@
       <c r="G107">
         <v>605</v>
       </c>
-      <c r="H107" t="s">
-        <v>67</v>
+      <c r="H107">
+        <v>0</v>
       </c>
       <c r="I107">
         <v>60.04</v>
@@ -6500,12 +6493,12 @@
         <v>1.556</v>
       </c>
       <c r="S107" s="6">
-        <f>(R107/(N107-O107))*100</f>
+        <f t="shared" si="8"/>
         <v>8.9409871861173364</v>
       </c>
     </row>
     <row r="108" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A108" s="13">
+      <c r="A108">
         <v>20250826</v>
       </c>
       <c r="B108" t="s">
@@ -6526,8 +6519,8 @@
       <c r="G108">
         <v>606</v>
       </c>
-      <c r="H108" t="s">
-        <v>67</v>
+      <c r="H108">
+        <v>0</v>
       </c>
       <c r="I108">
         <v>66.59</v>
@@ -6563,12 +6556,12 @@
         <v>1.1869999999999998</v>
       </c>
       <c r="S108" s="6">
-        <f>(R108/(N108-O108))*100</f>
+        <f t="shared" si="8"/>
         <v>7.1991751576904406</v>
       </c>
     </row>
     <row r="109" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A109" s="13">
+      <c r="A109">
         <v>20250826</v>
       </c>
       <c r="B109" t="s">
@@ -6589,8 +6582,8 @@
       <c r="G109">
         <v>607</v>
       </c>
-      <c r="H109" t="s">
-        <v>67</v>
+      <c r="H109">
+        <v>0</v>
       </c>
       <c r="I109">
         <v>69.19</v>
@@ -6626,12 +6619,12 @@
         <v>1.7720000000000002</v>
       </c>
       <c r="S109" s="6">
-        <f>(R109/(N109-O109))*100</f>
+        <f t="shared" si="8"/>
         <v>9.5422724824986549</v>
       </c>
     </row>
     <row r="110" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A110" s="13">
+      <c r="A110">
         <v>20250826</v>
       </c>
       <c r="B110" t="s">
@@ -6652,8 +6645,8 @@
       <c r="G110">
         <v>608</v>
       </c>
-      <c r="H110" t="s">
-        <v>67</v>
+      <c r="H110">
+        <v>0</v>
       </c>
       <c r="I110">
         <v>57.82</v>
@@ -6665,11 +6658,11 @@
         <v>27.84</v>
       </c>
       <c r="L110">
-        <f t="shared" ref="L110:L120" si="6">K110/I110</f>
+        <f t="shared" ref="L110:L120" si="9">K110/I110</f>
         <v>0.48149429263230714</v>
       </c>
       <c r="M110">
-        <f t="shared" ref="M110:M120" si="7">J110/I110</f>
+        <f t="shared" ref="M110:M120" si="10">J110/I110</f>
         <v>0.91663784157730888</v>
       </c>
       <c r="N110">
@@ -6685,16 +6678,16 @@
         <v>3.492</v>
       </c>
       <c r="R110">
-        <f t="shared" ref="R110:R120" si="8">Q110-P110</f>
+        <f t="shared" ref="R110:R120" si="11">Q110-P110</f>
         <v>1.2439999999999998</v>
       </c>
       <c r="S110" s="6">
-        <f>(R110/(N110-O110))*100</f>
+        <f t="shared" si="8"/>
         <v>7.3753483132744382</v>
       </c>
     </row>
     <row r="111" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A111" s="13">
+      <c r="A111">
         <v>20250826</v>
       </c>
       <c r="B111" t="s">
@@ -6715,8 +6708,8 @@
       <c r="G111">
         <v>609</v>
       </c>
-      <c r="H111" t="s">
-        <v>67</v>
+      <c r="H111">
+        <v>0</v>
       </c>
       <c r="I111">
         <v>72.069999999999993</v>
@@ -6728,11 +6721,11 @@
         <v>27.21</v>
       </c>
       <c r="L111">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0.3775496045511309</v>
       </c>
       <c r="M111">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.78021368114333289</v>
       </c>
       <c r="N111">
@@ -6748,16 +6741,16 @@
         <v>4.2939999999999996</v>
       </c>
       <c r="R111">
+        <f t="shared" si="11"/>
+        <v>2.0219999999999998</v>
+      </c>
+      <c r="S111" s="6">
         <f t="shared" si="8"/>
-        <v>2.0219999999999998</v>
-      </c>
-      <c r="S111" s="6">
-        <f>(R111/(N111-O111))*100</f>
         <v>9.9336772291820203</v>
       </c>
     </row>
     <row r="112" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A112" s="13">
+      <c r="A112">
         <v>20250826</v>
       </c>
       <c r="B112" t="s">
@@ -6778,8 +6771,8 @@
       <c r="G112">
         <v>610</v>
       </c>
-      <c r="H112" t="s">
-        <v>67</v>
+      <c r="H112">
+        <v>0</v>
       </c>
       <c r="I112">
         <v>77.48</v>
@@ -6791,11 +6784,11 @@
         <v>28.9</v>
       </c>
       <c r="L112">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0.37299948373773872</v>
       </c>
       <c r="M112">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.73825503355704702</v>
       </c>
       <c r="N112">
@@ -6811,16 +6804,16 @@
         <v>3.7090000000000001</v>
       </c>
       <c r="R112">
+        <f t="shared" si="11"/>
+        <v>1.4870000000000001</v>
+      </c>
+      <c r="S112" s="6">
         <f t="shared" si="8"/>
-        <v>1.4870000000000001</v>
-      </c>
-      <c r="S112" s="6">
-        <f>(R112/(N112-O112))*100</f>
         <v>6.0109952300105087</v>
       </c>
     </row>
     <row r="113" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A113" s="13">
+      <c r="A113">
         <v>20250826</v>
       </c>
       <c r="B113" t="s">
@@ -6841,8 +6834,8 @@
       <c r="G113">
         <v>611</v>
       </c>
-      <c r="H113" t="s">
-        <v>67</v>
+      <c r="H113">
+        <v>0</v>
       </c>
       <c r="I113">
         <v>70.739999999999995</v>
@@ -6854,11 +6847,11 @@
         <v>25.03</v>
       </c>
       <c r="L113">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0.35383093016680806</v>
       </c>
       <c r="M113">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.74370935821317508</v>
       </c>
       <c r="N113">
@@ -6874,16 +6867,16 @@
         <v>3.3719999999999999</v>
       </c>
       <c r="R113">
+        <f t="shared" si="11"/>
+        <v>1.08</v>
+      </c>
+      <c r="S113" s="6">
         <f t="shared" si="8"/>
-        <v>1.08</v>
-      </c>
-      <c r="S113" s="6">
-        <f>(R113/(N113-O113))*100</f>
         <v>6.3604240282685502</v>
       </c>
     </row>
     <row r="114" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A114" s="13">
+      <c r="A114">
         <v>20250826</v>
       </c>
       <c r="B114" t="s">
@@ -6904,8 +6897,8 @@
       <c r="G114">
         <v>612</v>
       </c>
-      <c r="H114" t="s">
-        <v>67</v>
+      <c r="H114">
+        <v>0</v>
       </c>
       <c r="I114">
         <v>61.96</v>
@@ -6917,11 +6910,11 @@
         <v>23.23</v>
       </c>
       <c r="L114">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0.37491930277598451</v>
       </c>
       <c r="M114">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.82391865719819235</v>
       </c>
       <c r="N114">
@@ -6937,16 +6930,16 @@
         <v>3.202</v>
       </c>
       <c r="R114">
+        <f t="shared" si="11"/>
+        <v>0.96399999999999997</v>
+      </c>
+      <c r="S114" s="6">
         <f t="shared" si="8"/>
-        <v>0.96399999999999997</v>
-      </c>
-      <c r="S114" s="6">
-        <f>(R114/(N114-O114))*100</f>
         <v>6.970858341167113</v>
       </c>
     </row>
     <row r="115" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A115" s="13">
+      <c r="A115">
         <v>20250826</v>
       </c>
       <c r="B115" t="s">
@@ -6967,8 +6960,8 @@
       <c r="G115">
         <v>613</v>
       </c>
-      <c r="H115" t="s">
-        <v>67</v>
+      <c r="H115">
+        <v>0</v>
       </c>
       <c r="I115">
         <v>60.95</v>
@@ -6980,11 +6973,11 @@
         <v>23.8</v>
       </c>
       <c r="L115">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0.39048400328137817</v>
       </c>
       <c r="M115">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.8495488105004102</v>
       </c>
       <c r="N115">
@@ -7000,16 +6993,16 @@
         <v>3.3959999999999999</v>
       </c>
       <c r="R115">
+        <f t="shared" si="11"/>
+        <v>1.177</v>
+      </c>
+      <c r="S115" s="6">
         <f t="shared" si="8"/>
-        <v>1.177</v>
-      </c>
-      <c r="S115" s="6">
-        <f>(R115/(N115-O115))*100</f>
         <v>8.8763197586726967</v>
       </c>
     </row>
     <row r="116" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A116" s="13">
+      <c r="A116">
         <v>20250826</v>
       </c>
       <c r="B116" t="s">
@@ -7030,8 +7023,8 @@
       <c r="G116" s="4">
         <v>614</v>
       </c>
-      <c r="H116" t="s">
-        <v>67</v>
+      <c r="H116">
+        <v>0</v>
       </c>
       <c r="I116">
         <v>73.58</v>
@@ -7043,11 +7036,11 @@
         <v>27.01</v>
       </c>
       <c r="L116">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0.36708344658874698</v>
       </c>
       <c r="M116">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.66077738515901063</v>
       </c>
       <c r="N116">
@@ -7063,16 +7056,16 @@
         <v>4.2859999999999996</v>
       </c>
       <c r="R116">
+        <f t="shared" si="11"/>
+        <v>2.0709999999999997</v>
+      </c>
+      <c r="S116" s="6">
         <f t="shared" si="8"/>
-        <v>2.0709999999999997</v>
-      </c>
-      <c r="S116" s="6">
-        <f>(R116/(N116-O116))*100</f>
         <v>10.408081214192379</v>
       </c>
     </row>
     <row r="117" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A117" s="13">
+      <c r="A117">
         <v>20250826</v>
       </c>
       <c r="B117" t="s">
@@ -7093,8 +7086,8 @@
       <c r="G117" s="4">
         <v>616</v>
       </c>
-      <c r="H117" t="s">
-        <v>67</v>
+      <c r="H117">
+        <v>0</v>
       </c>
       <c r="I117">
         <v>55.03</v>
@@ -7106,11 +7099,11 @@
         <v>23.37</v>
       </c>
       <c r="L117">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0.42467744866436491</v>
       </c>
       <c r="M117">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.80610576049427585</v>
       </c>
       <c r="N117">
@@ -7126,16 +7119,16 @@
         <v>3.214</v>
       </c>
       <c r="R117">
+        <f t="shared" si="11"/>
+        <v>0.97399999999999975</v>
+      </c>
+      <c r="S117" s="6">
         <f t="shared" si="8"/>
-        <v>0.97399999999999975</v>
-      </c>
-      <c r="S117" s="6">
-        <f>(R117/(N117-O117))*100</f>
         <v>9.1011025976452959</v>
       </c>
     </row>
     <row r="118" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A118" s="13">
+      <c r="A118">
         <v>20250826</v>
       </c>
       <c r="B118" t="s">
@@ -7156,8 +7149,8 @@
       <c r="G118" s="4">
         <v>617</v>
       </c>
-      <c r="H118" t="s">
-        <v>67</v>
+      <c r="H118">
+        <v>0</v>
       </c>
       <c r="I118">
         <v>61.09</v>
@@ -7169,11 +7162,11 @@
         <v>26.51</v>
       </c>
       <c r="L118">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0.43394990996889837</v>
       </c>
       <c r="M118">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.74480275004092322</v>
       </c>
       <c r="N118">
@@ -7189,16 +7182,16 @@
         <v>3.7290000000000001</v>
       </c>
       <c r="R118">
+        <f t="shared" si="11"/>
+        <v>1.4540000000000002</v>
+      </c>
+      <c r="S118" s="6">
         <f t="shared" si="8"/>
-        <v>1.4540000000000002</v>
-      </c>
-      <c r="S118" s="6">
-        <f>(R118/(N118-O118))*100</f>
         <v>12.032439589539893</v>
       </c>
     </row>
     <row r="119" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A119" s="13">
+      <c r="A119">
         <v>20250826</v>
       </c>
       <c r="B119" t="s">
@@ -7219,8 +7212,8 @@
       <c r="G119" s="4">
         <v>618</v>
       </c>
-      <c r="H119" t="s">
-        <v>67</v>
+      <c r="H119">
+        <v>0</v>
       </c>
       <c r="I119">
         <v>50.42</v>
@@ -7232,11 +7225,11 @@
         <v>18.07</v>
       </c>
       <c r="L119">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0.35838952796509321</v>
       </c>
       <c r="M119">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.66759222530741757</v>
       </c>
       <c r="N119">
@@ -7252,16 +7245,16 @@
         <v>2.5030000000000001</v>
       </c>
       <c r="R119">
+        <f t="shared" si="11"/>
+        <v>0.28699999999999992</v>
+      </c>
+      <c r="S119" s="6">
         <f t="shared" si="8"/>
-        <v>0.28699999999999992</v>
-      </c>
-      <c r="S119" s="6">
-        <f>(R119/(N119-O119))*100</f>
         <v>6.2134661182074034</v>
       </c>
     </row>
     <row r="120" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A120" s="13">
+      <c r="A120">
         <v>20250826</v>
       </c>
       <c r="B120" t="s">
@@ -7282,8 +7275,8 @@
       <c r="G120" s="4">
         <v>615</v>
       </c>
-      <c r="H120" t="s">
-        <v>67</v>
+      <c r="H120">
+        <v>0</v>
       </c>
       <c r="I120">
         <v>66.88</v>
@@ -7295,11 +7288,11 @@
         <v>28.93</v>
       </c>
       <c r="L120">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0.43256578947368424</v>
       </c>
       <c r="M120">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.75627990430622016</v>
       </c>
       <c r="N120">
@@ -7315,11 +7308,11 @@
         <v>4.12</v>
       </c>
       <c r="R120">
+        <f t="shared" si="11"/>
+        <v>1.9090000000000003</v>
+      </c>
+      <c r="S120" s="6">
         <f t="shared" si="8"/>
-        <v>1.9090000000000003</v>
-      </c>
-      <c r="S120" s="6">
-        <f>(R120/(N120-O120))*100</f>
         <v>12.404964585093254</v>
       </c>
       <c r="T120" t="s">
@@ -7327,7 +7320,7 @@
       </c>
     </row>
     <row r="121" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A121" s="13">
+      <c r="A121">
         <v>20250826</v>
       </c>
       <c r="B121" t="s">
@@ -7350,7 +7343,7 @@
       </c>
     </row>
     <row r="122" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A122" s="13">
+      <c r="A122">
         <v>20250826</v>
       </c>
       <c r="B122" t="s">
@@ -7371,8 +7364,8 @@
       <c r="G122">
         <v>619</v>
       </c>
-      <c r="H122" t="s">
-        <v>67</v>
+      <c r="H122">
+        <v>0</v>
       </c>
       <c r="I122">
         <v>59.23</v>
@@ -7413,7 +7406,7 @@
       </c>
     </row>
     <row r="123" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A123" s="13">
+      <c r="A123">
         <v>20250826</v>
       </c>
       <c r="B123" t="s">
@@ -7434,8 +7427,8 @@
       <c r="G123" s="4">
         <v>621</v>
       </c>
-      <c r="H123" t="s">
-        <v>67</v>
+      <c r="H123">
+        <v>0</v>
       </c>
       <c r="I123">
         <v>60.78</v>
@@ -7476,7 +7469,7 @@
       </c>
     </row>
     <row r="124" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A124" s="13">
+      <c r="A124">
         <v>20250826</v>
       </c>
       <c r="B124" t="s">
@@ -7497,8 +7490,8 @@
       <c r="G124" s="4">
         <v>620</v>
       </c>
-      <c r="H124" t="s">
-        <v>67</v>
+      <c r="H124">
+        <v>0</v>
       </c>
       <c r="I124">
         <v>74.05</v>
@@ -7539,7 +7532,7 @@
       </c>
     </row>
     <row r="125" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A125" s="13">
+      <c r="A125">
         <v>20250826</v>
       </c>
       <c r="B125" t="s">
@@ -7560,8 +7553,8 @@
       <c r="G125">
         <v>622</v>
       </c>
-      <c r="H125" t="s">
-        <v>67</v>
+      <c r="H125">
+        <v>0</v>
       </c>
       <c r="I125">
         <v>66.7</v>
@@ -7602,7 +7595,7 @@
       </c>
     </row>
     <row r="126" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A126" s="13">
+      <c r="A126">
         <v>20250826</v>
       </c>
       <c r="B126" t="s">
@@ -7623,8 +7616,8 @@
       <c r="G126">
         <v>623</v>
       </c>
-      <c r="H126" t="s">
-        <v>67</v>
+      <c r="H126">
+        <v>0</v>
       </c>
       <c r="I126">
         <v>62.73</v>
@@ -7665,7 +7658,7 @@
       </c>
     </row>
     <row r="127" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A127" s="13">
+      <c r="A127">
         <v>20250826</v>
       </c>
       <c r="B127" t="s">
@@ -7688,7 +7681,7 @@
       </c>
     </row>
     <row r="128" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A128" s="13">
+      <c r="A128">
         <v>20250826</v>
       </c>
       <c r="B128" t="s">
@@ -7709,15 +7702,15 @@
       <c r="G128">
         <v>624</v>
       </c>
-      <c r="H128" t="s">
-        <v>66</v>
+      <c r="H128">
+        <v>1</v>
       </c>
       <c r="I128" s="1">
         <v>82.13</v>
       </c>
     </row>
     <row r="129" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A129" s="13">
+      <c r="A129">
         <v>20250826</v>
       </c>
       <c r="B129" t="s">
@@ -7738,8 +7731,8 @@
       <c r="G129">
         <v>625</v>
       </c>
-      <c r="H129" t="s">
-        <v>67</v>
+      <c r="H129">
+        <v>0</v>
       </c>
       <c r="I129">
         <v>80.2</v>
@@ -7780,7 +7773,7 @@
       </c>
     </row>
     <row r="130" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A130" s="13">
+      <c r="A130">
         <v>20250826</v>
       </c>
       <c r="B130" t="s">
@@ -7801,15 +7794,15 @@
       <c r="G130">
         <v>626</v>
       </c>
-      <c r="H130" t="s">
-        <v>66</v>
+      <c r="H130">
+        <v>1</v>
       </c>
       <c r="I130" s="1">
         <v>54.83</v>
       </c>
     </row>
     <row r="131" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A131" s="13">
+      <c r="A131">
         <v>20250826</v>
       </c>
       <c r="B131" t="s">
@@ -7833,7 +7826,7 @@
       <c r="H131" s="12"/>
     </row>
     <row r="132" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A132" s="13">
+      <c r="A132">
         <v>20250826</v>
       </c>
       <c r="B132" t="s">
@@ -7854,8 +7847,8 @@
       <c r="G132">
         <v>628</v>
       </c>
-      <c r="H132" t="s">
-        <v>67</v>
+      <c r="H132">
+        <v>0</v>
       </c>
       <c r="I132" s="5">
         <v>51.02</v>
@@ -7892,7 +7885,7 @@
       </c>
     </row>
     <row r="133" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A133" s="13">
+      <c r="A133">
         <v>20250826</v>
       </c>
       <c r="B133" t="s">
@@ -7913,15 +7906,15 @@
       <c r="G133">
         <v>629</v>
       </c>
-      <c r="H133" t="s">
-        <v>66</v>
+      <c r="H133">
+        <v>1</v>
       </c>
       <c r="I133">
         <v>69.11</v>
       </c>
     </row>
     <row r="134" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A134" s="13">
+      <c r="A134">
         <v>20250826</v>
       </c>
       <c r="B134" t="s">
@@ -7942,8 +7935,8 @@
       <c r="G134">
         <v>630</v>
       </c>
-      <c r="H134" t="s">
-        <v>67</v>
+      <c r="H134">
+        <v>0</v>
       </c>
       <c r="I134">
         <v>80.13</v>
@@ -7984,7 +7977,7 @@
       </c>
     </row>
     <row r="135" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A135" s="13">
+      <c r="A135">
         <v>20250826</v>
       </c>
       <c r="B135" t="s">
@@ -8005,15 +7998,15 @@
       <c r="G135">
         <v>631</v>
       </c>
-      <c r="H135" t="s">
-        <v>66</v>
+      <c r="H135">
+        <v>1</v>
       </c>
       <c r="I135">
         <v>70.59</v>
       </c>
     </row>
     <row r="136" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A136" s="13">
+      <c r="A136">
         <v>20250826</v>
       </c>
       <c r="B136" t="s">
@@ -8034,8 +8027,8 @@
       <c r="G136">
         <v>632</v>
       </c>
-      <c r="H136" t="s">
-        <v>67</v>
+      <c r="H136">
+        <v>0</v>
       </c>
       <c r="I136">
         <v>71.760000000000005</v>
@@ -8076,7 +8069,7 @@
       </c>
     </row>
     <row r="137" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A137" s="13">
+      <c r="A137">
         <v>20250826</v>
       </c>
       <c r="B137" t="s">
@@ -8097,8 +8090,8 @@
       <c r="G137">
         <v>633</v>
       </c>
-      <c r="H137" t="s">
-        <v>67</v>
+      <c r="H137">
+        <v>0</v>
       </c>
       <c r="I137">
         <v>63.96</v>
@@ -8139,7 +8132,7 @@
       </c>
     </row>
     <row r="138" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A138" s="13">
+      <c r="A138">
         <v>20250826</v>
       </c>
       <c r="B138" t="s">
@@ -8160,8 +8153,8 @@
       <c r="G138">
         <v>634</v>
       </c>
-      <c r="H138" t="s">
-        <v>67</v>
+      <c r="H138">
+        <v>0</v>
       </c>
       <c r="I138">
         <v>78.099999999999994</v>
@@ -8202,7 +8195,7 @@
       </c>
     </row>
     <row r="139" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A139" s="13">
+      <c r="A139">
         <v>20250826</v>
       </c>
       <c r="B139" t="s">
@@ -8223,8 +8216,8 @@
       <c r="G139">
         <v>635</v>
       </c>
-      <c r="H139" t="s">
-        <v>67</v>
+      <c r="H139">
+        <v>0</v>
       </c>
       <c r="I139">
         <v>75.19</v>
@@ -8265,7 +8258,7 @@
       </c>
     </row>
     <row r="140" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A140" s="13">
+      <c r="A140">
         <v>20250826</v>
       </c>
       <c r="B140" t="s">
@@ -8286,8 +8279,8 @@
       <c r="G140">
         <v>636</v>
       </c>
-      <c r="H140" t="s">
-        <v>67</v>
+      <c r="H140">
+        <v>0</v>
       </c>
       <c r="I140">
         <v>63.06</v>
@@ -8328,7 +8321,7 @@
       </c>
     </row>
     <row r="141" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A141" s="13">
+      <c r="A141">
         <v>20250826</v>
       </c>
       <c r="B141" t="s">
@@ -8349,12 +8342,12 @@
       <c r="G141">
         <v>637</v>
       </c>
-      <c r="H141" t="s">
-        <v>66</v>
+      <c r="H141">
+        <v>1</v>
       </c>
     </row>
     <row r="142" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A142" s="13">
+      <c r="A142">
         <v>20250826</v>
       </c>
       <c r="B142" t="s">
@@ -8375,15 +8368,15 @@
       <c r="G142">
         <v>638</v>
       </c>
-      <c r="H142" t="s">
-        <v>66</v>
+      <c r="H142">
+        <v>1</v>
       </c>
       <c r="I142" s="1">
         <v>63.14</v>
       </c>
     </row>
     <row r="143" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A143" s="13">
+      <c r="A143">
         <v>20250826</v>
       </c>
       <c r="B143" t="s">
@@ -8404,8 +8397,8 @@
       <c r="G143">
         <v>639</v>
       </c>
-      <c r="H143" t="s">
-        <v>67</v>
+      <c r="H143">
+        <v>0</v>
       </c>
       <c r="I143">
         <v>49.64</v>
@@ -8446,7 +8439,7 @@
       </c>
     </row>
     <row r="144" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A144" s="13">
+      <c r="A144">
         <v>20250826</v>
       </c>
       <c r="B144" t="s">
@@ -8467,8 +8460,8 @@
       <c r="G144">
         <v>640</v>
       </c>
-      <c r="H144" t="s">
-        <v>67</v>
+      <c r="H144">
+        <v>0</v>
       </c>
       <c r="I144">
         <v>53.18</v>
@@ -8509,7 +8502,7 @@
       </c>
     </row>
     <row r="145" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A145" s="13">
+      <c r="A145">
         <v>20250826</v>
       </c>
       <c r="B145" t="s">
@@ -8530,8 +8523,8 @@
       <c r="G145">
         <v>641</v>
       </c>
-      <c r="H145" t="s">
-        <v>67</v>
+      <c r="H145">
+        <v>0</v>
       </c>
       <c r="I145">
         <v>60.19</v>
@@ -8572,7 +8565,7 @@
       </c>
     </row>
     <row r="146" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A146" s="13">
+      <c r="A146">
         <v>20250826</v>
       </c>
       <c r="B146" t="s">
@@ -8593,8 +8586,8 @@
       <c r="G146">
         <v>642</v>
       </c>
-      <c r="H146" t="s">
-        <v>67</v>
+      <c r="H146">
+        <v>0</v>
       </c>
       <c r="I146">
         <v>81.44</v>
@@ -8635,7 +8628,7 @@
       </c>
     </row>
     <row r="147" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A147" s="13">
+      <c r="A147">
         <v>20250826</v>
       </c>
       <c r="B147" t="s">
@@ -8656,15 +8649,15 @@
       <c r="G147">
         <v>643</v>
       </c>
-      <c r="H147" t="s">
-        <v>66</v>
+      <c r="H147">
+        <v>1</v>
       </c>
       <c r="I147" s="1">
         <v>70.849999999999994</v>
       </c>
     </row>
     <row r="148" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A148" s="13">
+      <c r="A148">
         <v>20250826</v>
       </c>
       <c r="B148" t="s">
@@ -8685,8 +8678,8 @@
       <c r="G148">
         <v>644</v>
       </c>
-      <c r="H148" t="s">
-        <v>67</v>
+      <c r="H148">
+        <v>0</v>
       </c>
       <c r="I148">
         <v>77.180000000000007</v>
@@ -8727,7 +8720,7 @@
       </c>
     </row>
     <row r="149" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A149" s="13">
+      <c r="A149">
         <v>20250826</v>
       </c>
       <c r="B149" t="s">
@@ -8748,12 +8741,12 @@
       <c r="G149">
         <v>645</v>
       </c>
-      <c r="H149" t="s">
-        <v>66</v>
+      <c r="H149">
+        <v>1</v>
       </c>
     </row>
     <row r="150" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A150" s="13">
+      <c r="A150">
         <v>20250826</v>
       </c>
       <c r="B150" t="s">
@@ -8774,8 +8767,8 @@
       <c r="G150">
         <v>646</v>
       </c>
-      <c r="H150" t="s">
-        <v>67</v>
+      <c r="H150">
+        <v>0</v>
       </c>
       <c r="I150">
         <v>77.930000000000007</v>
@@ -8816,7 +8809,7 @@
       </c>
     </row>
     <row r="151" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A151" s="13">
+      <c r="A151">
         <v>20250826</v>
       </c>
       <c r="B151" t="s">
@@ -8840,7 +8833,7 @@
       <c r="H151" s="12"/>
     </row>
     <row r="152" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A152" s="13">
+      <c r="A152">
         <v>20250826</v>
       </c>
       <c r="B152" t="s">
@@ -8861,8 +8854,8 @@
       <c r="G152">
         <v>648</v>
       </c>
-      <c r="H152" t="s">
-        <v>67</v>
+      <c r="H152">
+        <v>0</v>
       </c>
       <c r="I152">
         <v>73.900000000000006</v>
@@ -8903,7 +8896,7 @@
       </c>
     </row>
     <row r="153" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A153" s="13">
+      <c r="A153">
         <v>20250826</v>
       </c>
       <c r="B153" t="s">
@@ -8924,8 +8917,8 @@
       <c r="G153">
         <v>649</v>
       </c>
-      <c r="H153" t="s">
-        <v>67</v>
+      <c r="H153">
+        <v>0</v>
       </c>
       <c r="I153">
         <v>55.37</v>
@@ -8966,7 +8959,7 @@
       </c>
     </row>
     <row r="154" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A154" s="13">
+      <c r="A154">
         <v>20250826</v>
       </c>
       <c r="B154" t="s">
@@ -8987,8 +8980,8 @@
       <c r="G154">
         <v>650</v>
       </c>
-      <c r="H154" t="s">
-        <v>67</v>
+      <c r="H154">
+        <v>0</v>
       </c>
       <c r="I154">
         <v>63.48</v>
@@ -9029,7 +9022,7 @@
       </c>
     </row>
     <row r="155" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A155" s="13">
+      <c r="A155">
         <v>20250826</v>
       </c>
       <c r="B155" t="s">
@@ -9050,8 +9043,8 @@
       <c r="G155">
         <v>651</v>
       </c>
-      <c r="H155" t="s">
-        <v>67</v>
+      <c r="H155">
+        <v>0</v>
       </c>
       <c r="I155">
         <v>71.31</v>
@@ -9092,7 +9085,7 @@
       </c>
     </row>
     <row r="156" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A156" s="13">
+      <c r="A156">
         <v>20250826</v>
       </c>
       <c r="B156" t="s">
@@ -9113,15 +9106,15 @@
       <c r="G156">
         <v>652</v>
       </c>
-      <c r="H156" t="s">
-        <v>66</v>
+      <c r="H156">
+        <v>1</v>
       </c>
       <c r="I156">
         <v>45.61</v>
       </c>
     </row>
     <row r="157" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A157" s="13">
+      <c r="A157">
         <v>20250826</v>
       </c>
       <c r="B157" t="s">
@@ -9142,8 +9135,8 @@
       <c r="G157">
         <v>653</v>
       </c>
-      <c r="H157" t="s">
-        <v>67</v>
+      <c r="H157">
+        <v>0</v>
       </c>
       <c r="I157">
         <v>60.37</v>
@@ -9184,7 +9177,7 @@
       </c>
     </row>
     <row r="158" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A158" s="13">
+      <c r="A158">
         <v>20250826</v>
       </c>
       <c r="B158" t="s">
@@ -9205,8 +9198,8 @@
       <c r="G158">
         <v>654</v>
       </c>
-      <c r="H158" t="s">
-        <v>67</v>
+      <c r="H158">
+        <v>0</v>
       </c>
       <c r="I158">
         <v>69.8</v>
@@ -9247,7 +9240,7 @@
       </c>
     </row>
     <row r="159" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A159" s="13">
+      <c r="A159">
         <v>20250826</v>
       </c>
       <c r="B159" t="s">
@@ -9268,8 +9261,8 @@
       <c r="G159">
         <v>655</v>
       </c>
-      <c r="H159" t="s">
-        <v>67</v>
+      <c r="H159">
+        <v>0</v>
       </c>
       <c r="I159">
         <v>65.87</v>
@@ -9310,7 +9303,7 @@
       </c>
     </row>
     <row r="160" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A160" s="13">
+      <c r="A160">
         <v>20250826</v>
       </c>
       <c r="B160" t="s">
@@ -9331,12 +9324,12 @@
       <c r="G160">
         <v>656</v>
       </c>
-      <c r="H160" t="s">
-        <v>66</v>
+      <c r="H160">
+        <v>1</v>
       </c>
     </row>
     <row r="161" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A161" s="13">
+      <c r="A161">
         <v>20250826</v>
       </c>
       <c r="B161" t="s">
@@ -9357,15 +9350,15 @@
       <c r="G161">
         <v>657</v>
       </c>
-      <c r="H161" t="s">
-        <v>66</v>
+      <c r="H161">
+        <v>1</v>
       </c>
       <c r="I161">
         <v>58.19</v>
       </c>
     </row>
     <row r="162" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A162" s="13">
+      <c r="A162">
         <v>20250826</v>
       </c>
       <c r="B162" t="s">
@@ -9386,8 +9379,8 @@
       <c r="G162">
         <v>658</v>
       </c>
-      <c r="H162" t="s">
-        <v>67</v>
+      <c r="H162">
+        <v>0</v>
       </c>
       <c r="I162">
         <v>74.42</v>
@@ -9428,7 +9421,7 @@
       </c>
     </row>
     <row r="163" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A163" s="13">
+      <c r="A163">
         <v>20250826</v>
       </c>
       <c r="B163" t="s">
@@ -9449,8 +9442,8 @@
       <c r="G163">
         <v>659</v>
       </c>
-      <c r="H163" t="s">
-        <v>66</v>
+      <c r="H163">
+        <v>1</v>
       </c>
       <c r="I163">
         <v>53.31</v>
@@ -9460,7 +9453,7 @@
       </c>
     </row>
     <row r="164" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A164" s="13">
+      <c r="A164">
         <v>20250826</v>
       </c>
       <c r="B164" t="s">
@@ -9481,8 +9474,8 @@
       <c r="G164">
         <v>660</v>
       </c>
-      <c r="H164" t="s">
-        <v>67</v>
+      <c r="H164">
+        <v>0</v>
       </c>
       <c r="I164">
         <v>57.01</v>
@@ -9523,7 +9516,7 @@
       </c>
     </row>
     <row r="165" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A165" s="13">
+      <c r="A165">
         <v>20250826</v>
       </c>
       <c r="B165" t="s">
@@ -9544,8 +9537,8 @@
       <c r="G165">
         <v>661</v>
       </c>
-      <c r="H165" t="s">
-        <v>67</v>
+      <c r="H165">
+        <v>0</v>
       </c>
       <c r="I165">
         <v>63.69</v>
@@ -9586,7 +9579,7 @@
       </c>
     </row>
     <row r="166" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A166" s="13">
+      <c r="A166">
         <v>20250826</v>
       </c>
       <c r="B166" t="s">
@@ -9610,7 +9603,7 @@
       <c r="H166" s="12"/>
     </row>
     <row r="167" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A167" s="13">
+      <c r="A167">
         <v>20250826</v>
       </c>
       <c r="B167" t="s">
@@ -9631,8 +9624,8 @@
       <c r="G167">
         <v>663</v>
       </c>
-      <c r="H167" t="s">
-        <v>67</v>
+      <c r="H167">
+        <v>0</v>
       </c>
       <c r="I167">
         <v>65.17</v>
@@ -9673,7 +9666,7 @@
       </c>
     </row>
     <row r="168" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A168" s="13">
+      <c r="A168">
         <v>20250826</v>
       </c>
       <c r="B168" t="s">
@@ -9694,8 +9687,8 @@
       <c r="G168">
         <v>664</v>
       </c>
-      <c r="H168" t="s">
-        <v>67</v>
+      <c r="H168">
+        <v>0</v>
       </c>
       <c r="I168">
         <v>57.38</v>
@@ -9736,7 +9729,7 @@
       </c>
     </row>
     <row r="169" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A169" s="13">
+      <c r="A169">
         <v>20250826</v>
       </c>
       <c r="B169" t="s">
@@ -9757,8 +9750,8 @@
       <c r="G169">
         <v>665</v>
       </c>
-      <c r="H169" t="s">
-        <v>67</v>
+      <c r="H169">
+        <v>0</v>
       </c>
       <c r="I169">
         <v>59.77</v>

</xml_diff>